<commit_message>
feat(saff-study): publish specification and test suite v1.3
</commit_message>
<xml_diff>
--- a/output/xlsx/CRUDDocumentos--GT-.xlsx
+++ b/output/xlsx/CRUDDocumentos--GT-.xlsx
@@ -107,10 +107,10 @@
     <t>exibe lista completa de documentos</t>
   </si>
   <si>
-    <t>system: SYSTEM: exibe página com campos de cadastro de novo documento</t>
-  </si>
-  <si>
-    <t>exibe página com campos de cadastro de novo documento</t>
+    <t>system: SYSTEM: exibe pagina com campos de cadastro de novo documento</t>
+  </si>
+  <si>
+    <t>exibe pagina com campos de cadastro de novo documento</t>
   </si>
   <si>
     <t>system: SYSTEM: exibe lista de documentos</t>
@@ -137,10 +137,10 @@
     <t>exibe dados do documento</t>
   </si>
   <si>
-    <t>system: SYSTEM: se existir extração da familia cadastrada, esta deve exibir no campo Document um link para o novo documento</t>
-  </si>
-  <si>
-    <t>se existir extração da familia cadastrada, esta deve exibir no campo Document um link para o novo documento</t>
+    <t>system: SYSTEM: se existir extracao da familia cadastrada, esta deve exibir no campo Document um link para o novo documento</t>
+  </si>
+  <si>
+    <t>se existir extracao da familia cadastrada, esta deve exibir no campo Document um link para o novo documento</t>
   </si>
   <si>
     <t xml:space="preserve">Postcondition: </t>

</xml_diff>